<commit_message>
fix: Eliminate artificial sentence chunking and restore natural human sentence flow
</commit_message>
<xml_diff>
--- a/output/final_doc/What Happens to Expired or Rejected Medicines_quality_markers.xlsx
+++ b/output/final_doc/What Happens to Expired or Rejected Medicines_quality_markers.xlsx
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1692</v>
+        <v>1275</v>
       </c>
     </row>
     <row r="5">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -514,7 +514,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8.72713129296962</v>
+        <v>12.75543902633679</v>
       </c>
     </row>
     <row r="9">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>41.67390311968657</v>
+        <v>25.92981935355149</v>
       </c>
     </row>
   </sheetData>
@@ -571,15 +571,15 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>PASSED [✔]</t>
+          <t>FAILED [✘]</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>0.642798353909465</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Article body word count (FAQs excluded): 1205 words (Target: 1215 ± 100). Allowed range: [1115, 1315].</t>
+          <t>Article body word count (FAQs excluded): 781 words (Target: 1215 ± 100). Allowed range: [1115, 1315].</t>
         </is>
       </c>
     </row>
@@ -591,15 +591,15 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PASSED [✔]</t>
+          <t>FAILED [✘]</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Flesch Reading Ease: 41.7 (Target &gt;= 45+). Flesch-Kincaid Grade: 8.7 (Target &lt;= 8.5, Indian Grade 8).</t>
+          <t>Flesch Reading Ease: 25.9 (Target &gt;= 45+). Flesch-Kincaid Grade: 12.8 (Target &lt;= 8.5, Indian Grade 8).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Implement 4-Version editorial workflow with Version 4 reconstructed 100% locally in Python (0 LLM calls)
</commit_message>
<xml_diff>
--- a/output/final_doc/What Happens to Expired or Rejected Medicines_quality_markers.xlsx
+++ b/output/final_doc/What Happens to Expired or Rejected Medicines_quality_markers.xlsx
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1275</v>
+        <v>1271</v>
       </c>
     </row>
     <row r="5">
@@ -514,7 +514,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>12.75543902633679</v>
+        <v>12.56491284526683</v>
       </c>
     </row>
     <row r="9">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>25.92981935355149</v>
+        <v>27.34131223741846</v>
       </c>
     </row>
   </sheetData>
@@ -575,11 +575,11 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.642798353909465</v>
+        <v>0.6395061728395062</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Article body word count (FAQs excluded): 781 words (Target: 1215 ± 100). Allowed range: [1115, 1315].</t>
+          <t>Article body word count (FAQs excluded): 777 words (Target: 1215 ± 100). Allowed range: [1115, 1315].</t>
         </is>
       </c>
     </row>
@@ -599,7 +599,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Flesch Reading Ease: 25.9 (Target &gt;= 45+). Flesch-Kincaid Grade: 12.8 (Target &lt;= 8.5, Indian Grade 8).</t>
+          <t>Flesch Reading Ease: 27.3 (Target &gt;= 45+). Flesch-Kincaid Grade: 12.6 (Target &lt;= 8.5, Indian Grade 8).</t>
         </is>
       </c>
     </row>

</xml_diff>